<commit_message>
Fix OpenXML string tags and add CSV exports for Google Sheets compatibility
</commit_message>
<xml_diff>
--- a/reports/load_report.xlsx
+++ b/reports/load_report.xlsx
@@ -51,109 +51,83 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t>Metric</t>
-        </is>
+      <c r="A1" t="str" s="1">
+        <v>Metric</v>
       </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="B1" t="str" s="1">
+        <v>Value</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
+      <c r="A2" t="str">
+        <v>status</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
+      <c r="B2" t="str">
+        <v>PASSED</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>total_scenarios</t>
-        </is>
+      <c r="A3" t="str">
+        <v>total_scenarios</v>
       </c>
       <c r="B3" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>errors</t>
-        </is>
+      <c r="A4" t="str">
+        <v>errors</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>throughput_rps</t>
-        </is>
+      <c r="A5" t="str">
+        <v>throughput_rps</v>
       </c>
       <c r="B5" t="n">
         <v>4850</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>peak_virtual_users</t>
-        </is>
+      <c r="A6" t="str">
+        <v>peak_virtual_users</v>
       </c>
       <c r="B6" t="n">
         <v>5300</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>average_response_time_ms</t>
-        </is>
+      <c r="A7" t="str">
+        <v>average_response_time_ms</v>
       </c>
       <c r="B7" t="n">
         <v>28.4</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>failed</t>
-        </is>
+      <c r="A8" t="str">
+        <v>failed</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
+      <c r="A9" t="str">
+        <v>passed</v>
       </c>
       <c r="B9" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>suite</t>
-        </is>
+      <c r="A10" t="str">
+        <v>suite</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>TravelSync Load &amp; Stress Testing Suite</t>
-        </is>
+      <c r="B10" t="str">
+        <v>TravelSync Load &amp; Stress Testing Suite</v>
       </c>
     </row>
   </sheetData>

</xml_diff>